<commit_message>
Actualizar Informe_Commits_Ingecon con hashes y commits 76-77
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Incremento 3/Informe_Commits_Ingecon.xlsx
+++ b/Incremento 3/Informe_Commits_Ingecon.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codigo" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Documentos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Codigo" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Documentos" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -4309,7 +4309,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="B2:N80"/>
+  <dimension ref="B2:N82"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="2.43" customWidth="1" style="12" min="1" max="1"/>
@@ -4414,7 +4414,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E5" s="17" t="n"/>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>1b85769</t>
+        </is>
+      </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
           <t>Estructura inicial</t>
@@ -4463,7 +4467,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E6" s="20" t="n"/>
+      <c r="E6" s="20" t="inlineStr">
+        <is>
+          <t>b10a6a8</t>
+        </is>
+      </c>
       <c r="F6" s="21" t="inlineStr">
         <is>
           <t>Agregar carpetas vacías con .gitkeep</t>
@@ -4512,7 +4520,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E7" s="17" t="n"/>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>78fb80d</t>
+        </is>
+      </c>
       <c r="F7" s="18" t="inlineStr">
         <is>
           <t>Eliminar carpeta incremento_1</t>
@@ -4561,7 +4573,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E8" s="20" t="n"/>
+      <c r="E8" s="20" t="inlineStr">
+        <is>
+          <t>eaa6823</t>
+        </is>
+      </c>
       <c r="F8" s="21" t="inlineStr">
         <is>
           <t>Actualizar scripts de base de datos</t>
@@ -4610,7 +4626,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E9" s="17" t="n"/>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>a863d04</t>
+        </is>
+      </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
           <t>Actualizar scripts de base de datos</t>
@@ -4659,7 +4679,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E10" s="20" t="n"/>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>ecc79a4</t>
+        </is>
+      </c>
       <c r="F10" s="21" t="inlineStr">
         <is>
           <t>Actualización automática: 05/25/2026 19:34:43</t>
@@ -4708,7 +4732,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E11" s="17" t="n"/>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>8a2b897</t>
+        </is>
+      </c>
       <c r="F11" s="18" t="inlineStr">
         <is>
           <t>Delete ~$Carta_Gantt.xlsx</t>
@@ -4757,7 +4785,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E12" s="20" t="n"/>
+      <c r="E12" s="20" t="inlineStr">
+        <is>
+          <t>874900b</t>
+        </is>
+      </c>
       <c r="F12" s="21" t="inlineStr">
         <is>
           <t>Delete ~$Seguimiento_Sprint.xlsx</t>
@@ -4806,7 +4838,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E13" s="17" t="n"/>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>e9011f2</t>
+        </is>
+      </c>
       <c r="F13" s="18" t="inlineStr">
         <is>
           <t>Delete ~$matriz_RF_vs_CU.xlsx</t>
@@ -4855,7 +4891,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E14" s="20" t="n"/>
+      <c r="E14" s="20" t="inlineStr">
+        <is>
+          <t>436bd35</t>
+        </is>
+      </c>
       <c r="F14" s="21" t="inlineStr">
         <is>
           <t>Delete Documento_0_Grupo12.docx</t>
@@ -4904,7 +4944,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E15" s="17" t="n"/>
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>1935e8b</t>
+        </is>
+      </c>
       <c r="F15" s="18" t="inlineStr">
         <is>
           <t>Delete Dimensión Técnica Ingecon.docx</t>
@@ -4953,7 +4997,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E16" s="20" t="n"/>
+      <c r="E16" s="20" t="inlineStr">
+        <is>
+          <t>88ff908</t>
+        </is>
+      </c>
       <c r="F16" s="21" t="inlineStr">
         <is>
           <t>Delete Estimacion_Costos_y Beneficios.xlsx</t>
@@ -5002,7 +5050,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E17" s="17" t="n"/>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>2b29d67</t>
+        </is>
+      </c>
       <c r="F17" s="18" t="inlineStr">
         <is>
           <t>Delete Bizagi_Ingecon_Fases.bpm</t>
@@ -5051,7 +5103,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E18" s="20" t="n"/>
+      <c r="E18" s="20" t="inlineStr">
+        <is>
+          <t>82fd026</t>
+        </is>
+      </c>
       <c r="F18" s="21" t="inlineStr">
         <is>
           <t>Delete Carta_Gantt.xlsx</t>
@@ -5100,7 +5156,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E19" s="17" t="n"/>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>5cceffe</t>
+        </is>
+      </c>
       <c r="F19" s="18" t="inlineStr">
         <is>
           <t>Delete Seguimiento_Sprint.xlsx</t>
@@ -5149,7 +5209,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E20" s="20" t="n"/>
+      <c r="E20" s="20" t="inlineStr">
+        <is>
+          <t>05c6347</t>
+        </is>
+      </c>
       <c r="F20" s="21" t="inlineStr">
         <is>
           <t>Delete matriz_RF_vs_CU.xlsx</t>
@@ -5198,7 +5262,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E21" s="17" t="n"/>
+      <c r="E21" s="17" t="inlineStr">
+        <is>
+          <t>813f7cf</t>
+        </is>
+      </c>
       <c r="F21" s="18" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -5247,7 +5315,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E22" s="20" t="n"/>
+      <c r="E22" s="20" t="inlineStr">
+        <is>
+          <t>9973c25</t>
+        </is>
+      </c>
       <c r="F22" s="21" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -5296,7 +5368,11 @@
           <t>Diego Sepulveda</t>
         </is>
       </c>
-      <c r="E23" s="17" t="n"/>
+      <c r="E23" s="17" t="inlineStr">
+        <is>
+          <t>3076785</t>
+        </is>
+      </c>
       <c r="F23" s="18" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -5345,7 +5421,11 @@
           <t>Diego Sepulveda</t>
         </is>
       </c>
-      <c r="E24" s="20" t="n"/>
+      <c r="E24" s="20" t="inlineStr">
+        <is>
+          <t>2f49857</t>
+        </is>
+      </c>
       <c r="F24" s="21" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -5394,7 +5474,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E25" s="17" t="n"/>
+      <c r="E25" s="17" t="inlineStr">
+        <is>
+          <t>d6bb07b</t>
+        </is>
+      </c>
       <c r="F25" s="18" t="inlineStr">
         <is>
           <t>Se agrego el link del video de la presentacion</t>
@@ -5443,7 +5527,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E26" s="20" t="n"/>
+      <c r="E26" s="20" t="inlineStr">
+        <is>
+          <t>3cdf35d</t>
+        </is>
+      </c>
       <c r="F26" s="21" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -5492,7 +5580,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E27" s="17" t="n"/>
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>6ec78b1</t>
+        </is>
+      </c>
       <c r="F27" s="18" t="inlineStr">
         <is>
           <t>Create grabacion instalacion</t>
@@ -5541,7 +5633,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E28" s="20" t="n"/>
+      <c r="E28" s="20" t="inlineStr">
+        <is>
+          <t>05f4482</t>
+        </is>
+      </c>
       <c r="F28" s="21" t="inlineStr">
         <is>
           <t>Create instalacion windows</t>
@@ -5590,7 +5686,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E29" s="17" t="n"/>
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>3769096</t>
+        </is>
+      </c>
       <c r="F29" s="18" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -5639,7 +5739,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E30" s="20" t="n"/>
+      <c r="E30" s="20" t="inlineStr">
+        <is>
+          <t>1d0938e</t>
+        </is>
+      </c>
       <c r="F30" s="21" t="inlineStr">
         <is>
           <t>se agregaron links faltantes</t>
@@ -5688,7 +5792,11 @@
           <t>Diego Carabajal</t>
         </is>
       </c>
-      <c r="E31" s="17" t="n"/>
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>d67385f</t>
+        </is>
+      </c>
       <c r="F31" s="18" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -5737,7 +5845,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E32" s="20" t="n"/>
+      <c r="E32" s="20" t="inlineStr">
+        <is>
+          <t>8ac0b62</t>
+        </is>
+      </c>
       <c r="F32" s="21" t="inlineStr">
         <is>
           <t>se eliminaron links</t>
@@ -5786,7 +5898,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E33" s="17" t="n"/>
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>926ea16</t>
+        </is>
+      </c>
       <c r="F33" s="18" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -5835,7 +5951,11 @@
           <t>Diego Sepulveda</t>
         </is>
       </c>
-      <c r="E34" s="20" t="n"/>
+      <c r="E34" s="20" t="inlineStr">
+        <is>
+          <t>3ac7d85</t>
+        </is>
+      </c>
       <c r="F34" s="21" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -5884,7 +6004,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E35" s="17" t="n"/>
+      <c r="E35" s="17" t="inlineStr">
+        <is>
+          <t>d2cab6e</t>
+        </is>
+      </c>
       <c r="F35" s="18" t="inlineStr">
         <is>
           <t>Arreglos menores de gramatica</t>
@@ -5933,7 +6057,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E36" s="20" t="n"/>
+      <c r="E36" s="20" t="inlineStr">
+        <is>
+          <t>08c2b12</t>
+        </is>
+      </c>
       <c r="F36" s="21" t="inlineStr">
         <is>
           <t>Delete Bizagi_Ingecon_Final.bpm</t>
@@ -5982,7 +6110,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E37" s="17" t="n"/>
+      <c r="E37" s="17" t="inlineStr">
+        <is>
+          <t>b6abf4d</t>
+        </is>
+      </c>
       <c r="F37" s="18" t="inlineStr">
         <is>
           <t>Delete GUIA_INSTALACION_COMPLETA (1).pdf</t>
@@ -6031,7 +6163,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E38" s="20" t="n"/>
+      <c r="E38" s="20" t="inlineStr">
+        <is>
+          <t>a488313</t>
+        </is>
+      </c>
       <c r="F38" s="21" t="inlineStr">
         <is>
           <t>Delete Grupo 12 - Documento_0.docx</t>
@@ -6080,7 +6216,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E39" s="17" t="n"/>
+      <c r="E39" s="17" t="inlineStr">
+        <is>
+          <t>2950ddd</t>
+        </is>
+      </c>
       <c r="F39" s="18" t="inlineStr">
         <is>
           <t>Delete Grupo 12 - incremento1 .docx</t>
@@ -6129,7 +6269,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E40" s="20" t="n"/>
+      <c r="E40" s="20" t="inlineStr">
+        <is>
+          <t>74962d5</t>
+        </is>
+      </c>
       <c r="F40" s="21" t="inlineStr">
         <is>
           <t>Delete INFORME COMMITS.docx</t>
@@ -6178,7 +6322,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E41" s="17" t="n"/>
+      <c r="E41" s="17" t="inlineStr">
+        <is>
+          <t>2c17d58</t>
+        </is>
+      </c>
       <c r="F41" s="18" t="inlineStr">
         <is>
           <t>Delete MATRIZRF_CU.xlsx</t>
@@ -6227,7 +6375,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E42" s="20" t="n"/>
+      <c r="E42" s="20" t="inlineStr">
+        <is>
+          <t>51f3b89</t>
+        </is>
+      </c>
       <c r="F42" s="21" t="inlineStr">
         <is>
           <t>Delete Manual de usuario.pdf</t>
@@ -6276,7 +6428,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E43" s="17" t="n"/>
+      <c r="E43" s="17" t="inlineStr">
+        <is>
+          <t>f8b9af9</t>
+        </is>
+      </c>
       <c r="F43" s="18" t="inlineStr">
         <is>
           <t>Delete Presentacion Incremento 1</t>
@@ -6325,7 +6481,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E44" s="20" t="n"/>
+      <c r="E44" s="20" t="inlineStr">
+        <is>
+          <t>fdccb45</t>
+        </is>
+      </c>
       <c r="F44" s="21" t="inlineStr">
         <is>
           <t>Delete Seguimiento_Sprint (1).xlsx</t>
@@ -6374,7 +6534,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E45" s="17" t="n"/>
+      <c r="E45" s="17" t="inlineStr">
+        <is>
+          <t>affe874</t>
+        </is>
+      </c>
       <c r="F45" s="18" t="inlineStr">
         <is>
           <t>Delete grabacion instalacion</t>
@@ -6423,7 +6587,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E46" s="20" t="n"/>
+      <c r="E46" s="20" t="inlineStr">
+        <is>
+          <t>852af28</t>
+        </is>
+      </c>
       <c r="F46" s="21" t="inlineStr">
         <is>
           <t>Delete instalacion windows</t>
@@ -6472,7 +6640,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E47" s="17" t="n"/>
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>6222c69</t>
+        </is>
+      </c>
       <c r="F47" s="18" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -6521,7 +6693,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E48" s="20" t="n"/>
+      <c r="E48" s="20" t="inlineStr">
+        <is>
+          <t>e2b51f6</t>
+        </is>
+      </c>
       <c r="F48" s="21" t="inlineStr">
         <is>
           <t>Delete Documento 0/Documento 0 directory</t>
@@ -6570,7 +6746,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E49" s="17" t="n"/>
+      <c r="E49" s="17" t="inlineStr">
+        <is>
+          <t>bf9f9d7</t>
+        </is>
+      </c>
       <c r="F49" s="18" t="inlineStr">
         <is>
           <t>Create .gitkeep</t>
@@ -6619,7 +6799,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E50" s="20" t="n"/>
+      <c r="E50" s="20" t="inlineStr">
+        <is>
+          <t>5eb1f68</t>
+        </is>
+      </c>
       <c r="F50" s="21" t="inlineStr">
         <is>
           <t>Create .gitkeep</t>
@@ -6668,7 +6852,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E51" s="17" t="n"/>
+      <c r="E51" s="17" t="inlineStr">
+        <is>
+          <t>3670614</t>
+        </is>
+      </c>
       <c r="F51" s="18" t="inlineStr">
         <is>
           <t>Create .gitkeep</t>
@@ -6717,7 +6905,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E52" s="20" t="n"/>
+      <c r="E52" s="20" t="inlineStr">
+        <is>
+          <t>f68b487</t>
+        </is>
+      </c>
       <c r="F52" s="21" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -6766,7 +6958,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E53" s="17" t="n"/>
+      <c r="E53" s="17" t="inlineStr">
+        <is>
+          <t>4a60320</t>
+        </is>
+      </c>
       <c r="F53" s="18" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -6815,7 +7011,11 @@
           <t>Diego Carabajal</t>
         </is>
       </c>
-      <c r="E54" s="20" t="n"/>
+      <c r="E54" s="20" t="inlineStr">
+        <is>
+          <t>263bce1</t>
+        </is>
+      </c>
       <c r="F54" s="21" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -6864,7 +7064,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E55" s="17" t="n"/>
+      <c r="E55" s="17" t="inlineStr">
+        <is>
+          <t>4a17861</t>
+        </is>
+      </c>
       <c r="F55" s="18" t="inlineStr">
         <is>
           <t>Create .gitkeep</t>
@@ -6913,7 +7117,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E56" s="20" t="n"/>
+      <c r="E56" s="20" t="inlineStr">
+        <is>
+          <t>5c2a578</t>
+        </is>
+      </c>
       <c r="F56" s="21" t="inlineStr">
         <is>
           <t>Create .gitkeep</t>
@@ -6962,7 +7170,11 @@
           <t>Diego Carabajal</t>
         </is>
       </c>
-      <c r="E57" s="17" t="n"/>
+      <c r="E57" s="17" t="inlineStr">
+        <is>
+          <t>4d783aa</t>
+        </is>
+      </c>
       <c r="F57" s="18" t="inlineStr">
         <is>
           <t>Add installation files link to archivos.txt</t>
@@ -7011,7 +7223,11 @@
           <t>Diego Carabajal</t>
         </is>
       </c>
-      <c r="E58" s="20" t="n"/>
+      <c r="E58" s="20" t="inlineStr">
+        <is>
+          <t>8df5499</t>
+        </is>
+      </c>
       <c r="F58" s="21" t="inlineStr">
         <is>
           <t>Add link to external resource in codigo.txt</t>
@@ -7060,7 +7276,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E59" s="17" t="n"/>
+      <c r="E59" s="17" t="inlineStr">
+        <is>
+          <t>94aaf4e</t>
+        </is>
+      </c>
       <c r="F59" s="18" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -7109,7 +7329,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E60" s="20" t="n"/>
+      <c r="E60" s="20" t="inlineStr">
+        <is>
+          <t>f847766</t>
+        </is>
+      </c>
       <c r="F60" s="21" t="inlineStr">
         <is>
           <t>Add video links for project increments in README</t>
@@ -7158,7 +7382,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E61" s="17" t="n"/>
+      <c r="E61" s="17" t="inlineStr">
+        <is>
+          <t>38306d1</t>
+        </is>
+      </c>
       <c r="F61" s="18" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -7207,7 +7435,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E62" s="20" t="n"/>
+      <c r="E62" s="20" t="inlineStr">
+        <is>
+          <t>7d9efc5</t>
+        </is>
+      </c>
       <c r="F62" s="21" t="inlineStr">
         <is>
           <t>Delete Documento 0/Dimensión Técnica Ingecon.docx</t>
@@ -7256,7 +7488,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E63" s="17" t="n"/>
+      <c r="E63" s="17" t="inlineStr">
+        <is>
+          <t>1d8c68f</t>
+        </is>
+      </c>
       <c r="F63" s="18" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -7305,7 +7541,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E64" s="20" t="n"/>
+      <c r="E64" s="20" t="inlineStr">
+        <is>
+          <t>6d3980e</t>
+        </is>
+      </c>
       <c r="F64" s="21" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -7354,7 +7594,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E65" s="17" t="n"/>
+      <c r="E65" s="17" t="inlineStr">
+        <is>
+          <t>4308a03</t>
+        </is>
+      </c>
       <c r="F65" s="18" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -7403,7 +7647,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E66" s="20" t="n"/>
+      <c r="E66" s="20" t="inlineStr">
+        <is>
+          <t>839cfdd</t>
+        </is>
+      </c>
       <c r="F66" s="21" t="inlineStr">
         <is>
           <t>Delete Incremento 1/Diagramas_Secuencia.drawio</t>
@@ -7452,7 +7700,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E67" s="17" t="n"/>
+      <c r="E67" s="17" t="inlineStr">
+        <is>
+          <t>4561aeb</t>
+        </is>
+      </c>
       <c r="F67" s="18" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -7501,7 +7753,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E68" s="20" t="n"/>
+      <c r="E68" s="20" t="inlineStr">
+        <is>
+          <t>5acc2db</t>
+        </is>
+      </c>
       <c r="F68" s="21" t="inlineStr">
         <is>
           <t>Delete Incremento 2/Guia de Instalacion.pdf</t>
@@ -7550,7 +7806,11 @@
           <t>Paulina Urrutia</t>
         </is>
       </c>
-      <c r="E69" s="17" t="n"/>
+      <c r="E69" s="17" t="inlineStr">
+        <is>
+          <t>928e3cf</t>
+        </is>
+      </c>
       <c r="F69" s="18" t="inlineStr">
         <is>
           <t>Delete Incremento 1/Vista_lógica_BD.drawio</t>
@@ -7599,7 +7859,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E70" s="20" t="n"/>
+      <c r="E70" s="20" t="inlineStr">
+        <is>
+          <t>511e27b</t>
+        </is>
+      </c>
       <c r="F70" s="21" t="inlineStr">
         <is>
           <t>Update README to remove installation link</t>
@@ -7648,7 +7912,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E71" s="17" t="n"/>
+      <c r="E71" s="17" t="inlineStr">
+        <is>
+          <t>945093e</t>
+        </is>
+      </c>
       <c r="F71" s="18" t="inlineStr">
         <is>
           <t>Delete Incremento 1/Codigo directory</t>
@@ -7697,7 +7965,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E72" s="20" t="n"/>
+      <c r="E72" s="20" t="inlineStr">
+        <is>
+          <t>5a79b41</t>
+        </is>
+      </c>
       <c r="F72" s="21" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -7746,7 +8018,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E73" s="17" t="n"/>
+      <c r="E73" s="17" t="inlineStr">
+        <is>
+          <t>5cd0c0b</t>
+        </is>
+      </c>
       <c r="F73" s="18" t="inlineStr">
         <is>
           <t>Delete Incremento 1 directory</t>
@@ -7795,7 +8071,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E74" s="20" t="n"/>
+      <c r="E74" s="20" t="inlineStr">
+        <is>
+          <t>f1cd9ba</t>
+        </is>
+      </c>
       <c r="F74" s="21" t="inlineStr">
         <is>
           <t>Create .gitkeep</t>
@@ -7844,7 +8124,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E75" s="17" t="n"/>
+      <c r="E75" s="17" t="inlineStr">
+        <is>
+          <t>c269019</t>
+        </is>
+      </c>
       <c r="F75" s="18" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -7893,7 +8177,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E76" s="20" t="n"/>
+      <c r="E76" s="20" t="inlineStr">
+        <is>
+          <t>259cf90</t>
+        </is>
+      </c>
       <c r="F76" s="21" t="inlineStr">
         <is>
           <t>Add installation file link to archivos_instalacion.txt</t>
@@ -7942,7 +8230,11 @@
           <t>Diego Carabajal</t>
         </is>
       </c>
-      <c r="E77" s="17" t="n"/>
+      <c r="E77" s="17" t="inlineStr">
+        <is>
+          <t>e97ca33</t>
+        </is>
+      </c>
       <c r="F77" s="18" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -7991,7 +8283,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E78" s="20" t="n"/>
+      <c r="E78" s="20" t="inlineStr">
+        <is>
+          <t>86c5c29</t>
+        </is>
+      </c>
       <c r="F78" s="21" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -8040,7 +8336,11 @@
           <t>Vicente Ortega</t>
         </is>
       </c>
-      <c r="E79" s="17" t="n"/>
+      <c r="E79" s="17" t="inlineStr">
+        <is>
+          <t>d5ae6d4</t>
+        </is>
+      </c>
       <c r="F79" s="18" t="inlineStr">
         <is>
           <t>Add files via upload</t>
@@ -8075,40 +8375,146 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" ht="15" customHeight="1" s="13">
-      <c r="B80" s="22" t="inlineStr">
+    <row r="80" ht="28.35" customHeight="1" s="13">
+      <c r="B80" s="16" t="n">
+        <v>76</v>
+      </c>
+      <c r="C80" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-04 19:14</t>
+        </is>
+      </c>
+      <c r="D80" s="17" t="inlineStr">
+        <is>
+          <t>Vicente Ortega</t>
+        </is>
+      </c>
+      <c r="E80" s="17" t="inlineStr">
+        <is>
+          <t>5e7ce8d</t>
+        </is>
+      </c>
+      <c r="F80" s="18" t="inlineStr">
+        <is>
+          <t>Actualizar documentos de Documento 0 e Incrementos 1, 2 y 3</t>
+        </is>
+      </c>
+      <c r="G80" s="18" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="H80" s="18" t="inlineStr">
+        <is>
+          <t>Raiz y varios, Documento 0, Incremento 1, Incremento 2, Incremento 3</t>
+        </is>
+      </c>
+      <c r="I80" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="J80" s="16" t="n">
+        <v>14544</v>
+      </c>
+      <c r="K80" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="L80" s="16" t="n">
+        <v>29</v>
+      </c>
+      <c r="M80" s="16" t="n">
+        <v>14544</v>
+      </c>
+      <c r="N80" s="16" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="81" ht="28.35" customHeight="1" s="13">
+      <c r="B81" s="16" t="n">
+        <v>77</v>
+      </c>
+      <c r="C81" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-04 19:19</t>
+        </is>
+      </c>
+      <c r="D81" s="17" t="inlineStr">
+        <is>
+          <t>Vicente Ortega</t>
+        </is>
+      </c>
+      <c r="E81" s="17" t="inlineStr">
+        <is>
+          <t>455d401</t>
+        </is>
+      </c>
+      <c r="F81" s="18" t="inlineStr">
+        <is>
+          <t>Agregar carpetas ARCHIVOS NECESARIOS en Incrementos 1, 2 y 3</t>
+        </is>
+      </c>
+      <c r="G81" s="18" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="H81" s="18" t="inlineStr">
+        <is>
+          <t>Incremento 1, Incremento 2, Incremento 3</t>
+        </is>
+      </c>
+      <c r="I81" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="J81" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="K81" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L81" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="M81" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="N81" s="16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="82" ht="28.35" customHeight="1" s="13">
+      <c r="B82" s="22" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C80" s="23" t="n"/>
-      <c r="D80" s="23" t="n"/>
-      <c r="E80" s="23" t="n"/>
-      <c r="F80" s="23" t="n"/>
-      <c r="G80" s="23" t="n"/>
-      <c r="H80" s="23" t="n"/>
-      <c r="I80" s="24">
-        <f>SUM(I5:I79)</f>
+      <c r="C82" s="23" t="n"/>
+      <c r="D82" s="23" t="n"/>
+      <c r="E82" s="23" t="n"/>
+      <c r="F82" s="23" t="n"/>
+      <c r="G82" s="23" t="n"/>
+      <c r="H82" s="23" t="n"/>
+      <c r="I82" s="24">
+        <f>SUM(I5:I81)</f>
         <v/>
       </c>
-      <c r="J80" s="24">
-        <f>SUM(J5:J79)</f>
+      <c r="J82" s="24">
+        <f>SUM(J5:J81)</f>
         <v/>
       </c>
-      <c r="K80" s="24">
-        <f>SUM(K5:K79)</f>
+      <c r="K82" s="24">
+        <f>SUM(K5:K81)</f>
         <v/>
       </c>
-      <c r="L80" s="24">
-        <f>SUM(L5:L79)</f>
+      <c r="L82" s="24">
+        <f>SUM(L5:L81)</f>
         <v/>
       </c>
-      <c r="M80" s="24">
-        <f>SUM(M5:M79)</f>
+      <c r="M82" s="24">
+        <f>SUM(M5:M81)</f>
         <v/>
       </c>
-      <c r="N80" s="24">
-        <f>SUM(N5:N79)</f>
+      <c r="N82" s="24">
+        <f>SUM(N5:N81)</f>
         <v/>
       </c>
     </row>

</xml_diff>